<commit_message>
data: use lightweight licensed spot thumbnails
</commit_message>
<xml_diff>
--- a/exports/dia-diem-chup-anh-threads-aphoto-thang-10-2026.xlsx
+++ b/exports/dia-diem-chup-anh-threads-aphoto-thang-10-2026.xlsx
@@ -580,7 +580,7 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/b/b5/Chateau-eau-hang-dau-hanoi.jpg</t>
+          <t>https://thumb.wikimedia.org/wikipedia/commons/thumb/b/b5/Chateau-eau-hang-dau-hanoi.jpg/960px-Chateau-eau-hang-dau-hanoi.jpg</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -645,7 +645,7 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/b/b7/Main_gate_of_the_Temple_of_Literature%2C_Hanoi%2C_Vietnam%2C_20240123_0929_3068.jpg</t>
+          <t>https://thumb.wikimedia.org/wikipedia/commons/thumb/b/b7/Main_gate_of_the_Temple_of_Literature%2C_Hanoi%2C_Vietnam%2C_20240123_0929_3068.jpg/960px-Main_gate_of_the_Temple_of_Literature%2C_Hanoi%2C_Vietnam%2C_20240123_0929_3068.jpg</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -710,7 +710,7 @@
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/b/bd/Thong_Nhat_Park.jpg</t>
+          <t>https://thumb.wikimedia.org/wikipedia/commons/thumb/b/bd/Thong_Nhat_Park.jpg/960px-Thong_Nhat_Park.jpg</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -775,7 +775,7 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/a/af/St_Josephs_Cathedral_of_Hanoi.jpg</t>
+          <t>https://thumb.wikimedia.org/wikipedia/commons/thumb/a/af/St_Josephs_Cathedral_of_Hanoi.jpg/960px-St_Josephs_Cathedral_of_Hanoi.jpg</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -840,7 +840,7 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/7/75/Ph%E1%BB%91_H%C3%A0ng_M%C3%A3%2C_H%C3%A0_N%E1%BB%99i_001.JPG</t>
+          <t>https://thumb.wikimedia.org/wikipedia/commons/thumb/7/75/Ph%E1%BB%91_H%C3%A0ng_M%C3%A3%2C_H%C3%A0_N%E1%BB%99i_001.JPG/960px-Ph%E1%BB%91_H%C3%A0ng_M%C3%A3%2C_H%C3%A0_N%E1%BB%99i_001.JPG</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -905,7 +905,7 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/1/10/Ph%E1%BB%91_B%C3%ADch_H%E1%BB%8Da_Ph%C3%B9ng_H%C6%B0ng_H%C3%A0ng_M%C3%A3_Ho%C3%A0n_Ki%E1%BA%BFm_H%C3%A0_N%E1%BB%99i_Vietnam_%282%29.jpg</t>
+          <t>https://thumb.wikimedia.org/wikipedia/commons/thumb/1/10/Ph%E1%BB%91_B%C3%ADch_H%E1%BB%8Da_Ph%C3%B9ng_H%C6%B0ng_H%C3%A0ng_M%C3%A3_Ho%C3%A0n_Ki%E1%BA%BFm_H%C3%A0_N%E1%BB%99i_Vietnam_%282%29.jpg/960px-Ph%E1%BB%91_B%C3%ADch_H%E1%BB%8Da_Ph%C3%B9ng_H%C6%B0ng_H%C3%A0ng_M%C3%A3_Ho%C3%A0n_Ki%E1%BA%BFm_H%C3%A0_N%E1%BB%99i_Vietnam_%282%29.jpg</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -970,7 +970,7 @@
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/8/81/Hanoi_Botanical_Garden_%2820140802_173053%29.jpg</t>
+          <t>https://thumb.wikimedia.org/wikipedia/commons/thumb/8/81/Hanoi_Botanical_Garden_%2820140802_173053%29.jpg/960px-Hanoi_Botanical_Garden_%2820140802_173053%29.jpg</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/b/b5/Chateau-eau-hang-dau-hanoi.jpg</t>
+          <t>https://thumb.wikimedia.org/wikipedia/commons/thumb/b/b5/Chateau-eau-hang-dau-hanoi.jpg/960px-Chateau-eau-hang-dau-hanoi.jpg</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/b/b7/Main_gate_of_the_Temple_of_Literature%2C_Hanoi%2C_Vietnam%2C_20240123_0929_3068.jpg</t>
+          <t>https://thumb.wikimedia.org/wikipedia/commons/thumb/b/b7/Main_gate_of_the_Temple_of_Literature%2C_Hanoi%2C_Vietnam%2C_20240123_0929_3068.jpg/960px-Main_gate_of_the_Temple_of_Literature%2C_Hanoi%2C_Vietnam%2C_20240123_0929_3068.jpg</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/b/bd/Thong_Nhat_Park.jpg</t>
+          <t>https://thumb.wikimedia.org/wikipedia/commons/thumb/b/bd/Thong_Nhat_Park.jpg/960px-Thong_Nhat_Park.jpg</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1311,7 +1311,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/a/af/St_Josephs_Cathedral_of_Hanoi.jpg</t>
+          <t>https://thumb.wikimedia.org/wikipedia/commons/thumb/a/af/St_Josephs_Cathedral_of_Hanoi.jpg/960px-St_Josephs_Cathedral_of_Hanoi.jpg</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1363,7 +1363,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/7/75/Ph%E1%BB%91_H%C3%A0ng_M%C3%A3%2C_H%C3%A0_N%E1%BB%99i_001.JPG</t>
+          <t>https://thumb.wikimedia.org/wikipedia/commons/thumb/7/75/Ph%E1%BB%91_H%C3%A0ng_M%C3%A3%2C_H%C3%A0_N%E1%BB%99i_001.JPG/960px-Ph%E1%BB%91_H%C3%A0ng_M%C3%A3%2C_H%C3%A0_N%E1%BB%99i_001.JPG</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -1415,7 +1415,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/1/10/Ph%E1%BB%91_B%C3%ADch_H%E1%BB%8Da_Ph%C3%B9ng_H%C6%B0ng_H%C3%A0ng_M%C3%A3_Ho%C3%A0n_Ki%E1%BA%BFm_H%C3%A0_N%E1%BB%99i_Vietnam_%282%29.jpg</t>
+          <t>https://thumb.wikimedia.org/wikipedia/commons/thumb/1/10/Ph%E1%BB%91_B%C3%ADch_H%E1%BB%8Da_Ph%C3%B9ng_H%C6%B0ng_H%C3%A0ng_M%C3%A3_Ho%C3%A0n_Ki%E1%BA%BFm_H%C3%A0_N%E1%BB%99i_Vietnam_%282%29.jpg/960px-Ph%E1%BB%91_B%C3%ADch_H%E1%BB%8Da_Ph%C3%B9ng_H%C6%B0ng_H%C3%A0ng_M%C3%A3_Ho%C3%A0n_Ki%E1%BA%BFm_H%C3%A0_N%E1%BB%99i_Vietnam_%282%29.jpg</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/8/81/Hanoi_Botanical_Garden_%2820140802_173053%29.jpg</t>
+          <t>https://thumb.wikimedia.org/wikipedia/commons/thumb/8/81/Hanoi_Botanical_Garden_%2820140802_173053%29.jpg/960px-Hanoi_Botanical_Garden_%2820140802_173053%29.jpg</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">

</xml_diff>